<commit_message>
Update CaseStudy_Networks notebook and clean up generated case study files
</commit_message>
<xml_diff>
--- a/Energy_Italy/Hydro inflows 2017.xlsx
+++ b/Energy_Italy/Hydro inflows 2017.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BAKARY JAMMEH\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimibit-my.sharepoint.com/personal/b_jammeh_campus_unimib_it/Documents/Desktop/MODELLING/Italian_cge_model/AdOpT-NET0_Bakary/Energy_Italy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62C5FF5E-C9E6-46C8-A9BB-69EFC047BFA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{62C5FF5E-C9E6-46C8-A9BB-69EFC047BFA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1902A9D-1B98-49F3-BD75-B2F924AE95B0}"/>
   <bookViews>
-    <workbookView xWindow="20715" yWindow="3405" windowWidth="12855" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28350" yWindow="2985" windowWidth="10065" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="inflows" sheetId="2" r:id="rId1"/>
+    <sheet name="Hydro_inflows" sheetId="2" r:id="rId1"/>
     <sheet name="README" sheetId="1" r:id="rId2"/>
     <sheet name="MacroRegion_Totals" sheetId="3" r:id="rId3"/>
     <sheet name="Zone_Totals" sheetId="4" r:id="rId4"/>

</xml_diff>